<commit_message>
BWI sync — 2026-06-29 13:12 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Austria.xlsx
+++ b/BWI/bestwine_output/bestwine_Austria.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA865"/>
+  <dimension ref="A1:AA866"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -85892,6 +85892,99 @@
       <c r="Z865" s="2" t="inlineStr"/>
       <c r="AA865" s="2" t="inlineStr"/>
     </row>
+    <row r="866">
+      <c r="A866" s="2" t="inlineStr">
+        <is>
+          <t>Wein.depot Noitz</t>
+        </is>
+      </c>
+      <c r="B866" s="2" t="inlineStr">
+        <is>
+          <t>Wein.depot Noitz</t>
+        </is>
+      </c>
+      <c r="C866" s="2" t="inlineStr">
+        <is>
+          <t>692</t>
+        </is>
+      </c>
+      <c r="D866" s="2" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E866" s="2" t="inlineStr">
+        <is>
+          <t>Furth bei Göttweig</t>
+        </is>
+      </c>
+      <c r="F866" s="2" t="inlineStr">
+        <is>
+          <t>Lower Austria</t>
+        </is>
+      </c>
+      <c r="G866" s="2" t="inlineStr">
+        <is>
+          <t>169 Römerstraße</t>
+        </is>
+      </c>
+      <c r="H866" s="2" t="inlineStr">
+        <is>
+          <t>3511</t>
+        </is>
+      </c>
+      <c r="I866" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wein-handlung.at</t>
+        </is>
+      </c>
+      <c r="J866" s="2" t="inlineStr"/>
+      <c r="K866" s="2" t="inlineStr"/>
+      <c r="L866" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="M866" s="2" t="inlineStr"/>
+      <c r="N866" s="2" t="inlineStr">
+        <is>
+          <t>wein.depot@aon.at</t>
+        </is>
+      </c>
+      <c r="O866" s="2" t="inlineStr">
+        <is>
+          <t>+43 2732 85656</t>
+        </is>
+      </c>
+      <c r="P866" s="2" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="Q866" s="2" t="inlineStr">
+        <is>
+          <t>ATU61892946</t>
+        </is>
+      </c>
+      <c r="R866" s="2" t="inlineStr"/>
+      <c r="S866" s="2" t="inlineStr"/>
+      <c r="T866" s="2" t="inlineStr"/>
+      <c r="U866" s="2" t="inlineStr"/>
+      <c r="V866" s="2" t="inlineStr"/>
+      <c r="W866" s="2" t="inlineStr">
+        <is>
+          <t>Franz Noitz</t>
+        </is>
+      </c>
+      <c r="X866" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="Y866" s="2" t="inlineStr"/>
+      <c r="Z866" s="2" t="inlineStr"/>
+      <c r="AA866" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>